<commit_message>
Aggiornamento mappe autisti (auto-publish)
</commit_message>
<xml_diff>
--- a/AppLogSolutionLocale/dati/CONSEGNE/CONSEGNE_28-04-2026/punti_consegna.xlsx
+++ b/AppLogSolutionLocale/dati/CONSEGNE/CONSEGNE_28-04-2026/punti_consegna.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,20 +449,40 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Orario min Frutta</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Orario max Frutta</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Orario min Latte</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Orario max Latte</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Orario min</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Orario max</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Latitudine</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Longitudine</t>
         </is>
@@ -509,10 +529,30 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>45.67766254908982</v>
       </c>
-      <c r="J2" t="n">
+      <c r="N2" t="n">
         <v>12.10578351498602</v>
       </c>
     </row>
@@ -554,13 +594,25 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>45.30961682015293</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>12.07423983558196</v>
       </c>
     </row>
@@ -605,10 +657,30 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
         <v>45.19040334865818</v>
       </c>
-      <c r="J4" t="n">
+      <c r="N4" t="n">
         <v>12.04072566746522</v>
       </c>
     </row>

</xml_diff>